<commit_message>
delete leaf image, widen columns for threshold_p
</commit_message>
<xml_diff>
--- a/data/threshold_p.xlsx
+++ b/data/threshold_p.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Joe/Documents/College/02- R code/2- heating/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R\heat_tolerance\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DBBD99-32AA-BB45-A363-39EF159EBBFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C16AF16-2EAA-42C9-A033-D2D1D099BF6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15740" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25710" yWindow="375" windowWidth="24090" windowHeight="19200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="June_2022" sheetId="1" r:id="rId1"/>
@@ -512,12 +512,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="10" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="10" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -549,7 +553,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -581,7 +585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -613,7 +617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -645,7 +649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -677,7 +681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -709,7 +713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -741,7 +745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -773,7 +777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -805,7 +809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -837,7 +841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -869,7 +873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -909,12 +913,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -946,7 +959,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -978,7 +991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1010,7 +1023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1042,7 +1055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1074,7 +1087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1106,7 +1119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -1138,7 +1151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1170,7 +1183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1202,7 +1215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1234,7 +1247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1266,7 +1279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1306,12 +1319,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="13" width="15.5" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="13" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1352,7 +1368,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1393,7 +1409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1434,7 +1450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1475,7 +1491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1516,7 +1532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1557,7 +1573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -1598,7 +1614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1639,7 +1655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1680,7 +1696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1721,7 +1737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1762,7 +1778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1811,12 +1827,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="13" width="16" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="13" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1857,7 +1877,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1898,7 +1918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1939,7 +1959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1980,7 +2000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -2021,7 +2041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -2062,7 +2082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -2103,7 +2123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2144,7 +2164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -2185,7 +2205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -2226,7 +2246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -2267,7 +2287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -2316,12 +2336,21 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="10" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2353,7 +2382,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -2385,7 +2414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -2417,7 +2446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -2449,7 +2478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -2481,7 +2510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -2513,7 +2542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -2545,7 +2574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2577,7 +2606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -2609,7 +2638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -2641,7 +2670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -2673,7 +2702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>42</v>
       </c>

</xml_diff>

<commit_message>
adding back in boot 1000 file. Updating threshold testing.R to include critical threshold temperature against leaf temp. Update threshold_p table to reflect these new p values
</commit_message>
<xml_diff>
--- a/data/threshold_p.xlsx
+++ b/data/threshold_p.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R\heat_tolerance\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C16AF16-2EAA-42C9-A033-D2D1D099BF6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50BDF5F3-2082-4738-AFA5-464D8CA2E716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25710" yWindow="375" windowWidth="24090" windowHeight="19200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="510" yWindow="690" windowWidth="35265" windowHeight="19275" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="June_2022" sheetId="1" r:id="rId1"/>
@@ -18,13 +18,18 @@
     <sheet name="July_2022" sheetId="3" r:id="rId3"/>
     <sheet name="July_2023" sheetId="4" r:id="rId4"/>
     <sheet name="Sept_2023" sheetId="5" r:id="rId5"/>
+    <sheet name="leaf_June_2022" sheetId="7" r:id="rId6"/>
+    <sheet name="leaf_July_2022" sheetId="8" r:id="rId7"/>
+    <sheet name="leaf_June_2023" sheetId="9" r:id="rId8"/>
+    <sheet name="leaf_July_2023" sheetId="10" r:id="rId9"/>
+    <sheet name="Leaf temperature table" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="60">
   <si>
     <t>species</t>
   </si>
@@ -153,6 +158,57 @@
   </si>
   <si>
     <t>Ulmus rubra</t>
+  </si>
+  <si>
+    <t>Leaf June 22(tcrit)</t>
+  </si>
+  <si>
+    <t>Leaf June 22 (T50)</t>
+  </si>
+  <si>
+    <t>Leaf June 22 (T95)</t>
+  </si>
+  <si>
+    <t>Leaf July 22(tcrit)</t>
+  </si>
+  <si>
+    <t>Leaf July 22 (T50)</t>
+  </si>
+  <si>
+    <t>Leaf July 22 (T95)</t>
+  </si>
+  <si>
+    <t>Leaf June 23(tcrit)</t>
+  </si>
+  <si>
+    <t>Leaf June 23 (T50)</t>
+  </si>
+  <si>
+    <t>Leaf June 23 (T95)</t>
+  </si>
+  <si>
+    <t>Leaf July 23(tcrit)</t>
+  </si>
+  <si>
+    <t>Leaf July 23 (T50)</t>
+  </si>
+  <si>
+    <t>Leaf July 23 (T95)</t>
+  </si>
+  <si>
+    <t>Species</t>
+  </si>
+  <si>
+    <t>&lt;0.001</t>
+  </si>
+  <si>
+    <t>&gt;0.999</t>
+  </si>
+  <si>
+    <t>Leaf temperature 2022</t>
+  </si>
+  <si>
+    <t>Leaf temperature 2023</t>
   </si>
 </sst>
 </file>
@@ -510,15 +566,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11A23EA5-2325-434B-921E-4888F3AE2CCE}">
   <dimension ref="A1:J12"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="10" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="18.140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -903,6 +964,234 @@
       </c>
       <c r="J12">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEC6A3F6-6EE5-46A3-BDCC-C293A1205373}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0.50700000000000001</v>
+      </c>
+      <c r="G2">
+        <v>0.50509999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4">
+        <v>0.79200000000000004</v>
+      </c>
+      <c r="E4">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="F4">
+        <v>0.48</v>
+      </c>
+      <c r="G4">
+        <v>8.4000000000000005E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0.13730000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>1E-3</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>1E-3</v>
+      </c>
+      <c r="G6">
+        <v>1.4E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7">
+        <v>0.73899999999999999</v>
+      </c>
+      <c r="E7">
+        <v>0.62</v>
+      </c>
+      <c r="F7">
+        <v>0.996</v>
+      </c>
+      <c r="G7">
+        <v>0.98699999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0.5575</v>
+      </c>
+      <c r="G8">
+        <v>0.60760000000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="E9">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="F9">
+        <v>0.3206</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10">
+        <v>0.126</v>
+      </c>
+      <c r="E10">
+        <v>0.66</v>
+      </c>
+      <c r="F10" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10">
+        <v>0.22520000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11">
+        <v>0.16220000000000001</v>
+      </c>
+      <c r="E11">
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>0.996</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12">
+        <v>0.96679999999999999</v>
+      </c>
+      <c r="E12">
+        <v>0.22800000000000001</v>
+      </c>
+      <c r="F12">
+        <v>0.54449999999999998</v>
+      </c>
+      <c r="G12">
+        <v>0.252</v>
       </c>
     </row>
   </sheetData>
@@ -911,20 +1200,20 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D53B27CB-D8BB-4E46-ADAD-0AE8D850274C}">
   <dimension ref="A1:J12"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="18.140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -1317,14 +1606,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9D90E0E-E5C9-4C00-871A-58F89E091DCC}">
   <dimension ref="A1:M12"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="13" width="15.42578125" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="13" width="15.42578125" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1825,15 +2114,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1B08285-B35B-489F-81DD-B5CF4588D20B}">
   <dimension ref="A1:M12"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="13" width="16" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="13" width="16" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -2334,20 +2623,20 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF94F7A4-A0CB-421F-90FD-0E0386F20B78}">
   <dimension ref="A1:J12"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="24.85546875" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="4" max="4" width="21" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="24.28515625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="8" max="8" width="18.140625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="24.28515625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2737,4 +3026,731 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61FF9E2E-0CBB-41EF-B66E-C880883327CE}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>0.79200000000000004</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>1E-3</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>0.73899999999999999</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10">
+        <v>0.126</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11">
+        <v>0.16220000000000001</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12">
+        <v>0.96679999999999999</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82411354-F273-4155-8CD9-88615BC0F50E}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>0.62</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10">
+        <v>0.66</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11">
+        <v>0.24199999999999999</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12">
+        <v>0.22800000000000001</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16A93065-8F95-4CD1-98BD-E65F1389D409}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>0.50700000000000001</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>0.48</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>1E-3</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>0.996</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>0.5575</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>0.3206</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12">
+        <v>0.54449999999999998</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20164656-928B-4E0C-ACE5-CCF2597F73FF}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>0.50509999999999999</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>8.4000000000000005E-2</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>0.13730000000000001</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>1.4E-2</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>0.98699999999999999</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>0.60760000000000003</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10">
+        <v>0.22520000000000001</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11">
+        <v>0.996</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12">
+        <v>0.252</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>